<commit_message>
Data sweep: company names become roles (Owner, EPC, Engineer, Consultant), project number removed, Fimiston becomes FIM, Gidji the offsite roaster; tools/sanitize.py keeps it that way after rebuilds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KTEDhnU5tNU91Jmkwz9aQB
</commit_message>
<xml_diff>
--- a/sources/cp1.xlsx
+++ b/sources/cp1.xlsx
@@ -702,7 +702,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Process Control Philosophy KCGM Enabling Works – Stage 1</t>
+          <t>Process Control Philosophy Owner Enabling Works – Stage 1</t>
         </is>
       </c>
     </row>
@@ -1836,12 +1836,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>KCGM</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Kalgoorlie Consolidated Gold Mines</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1884,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NSR</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Northern Star Resources Ltd</t>
+          <t>Owner</t>
         </is>
       </c>
     </row>

</xml_diff>